<commit_message>
Updated to have sentiment filter
</commit_message>
<xml_diff>
--- a/dist/private_credit_stress.xlsx
+++ b/dist/private_credit_stress.xlsx
@@ -532,22 +532,18 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Partners Group</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>PGHN</t>
-        </is>
-      </c>
+          <t>Marblegate Asset Management</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n">
-        <v>62.96</v>
+        <v>87.78</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -556,7 +552,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>lender_nav_stability</t>
+          <t>lender_spread_power</t>
         </is>
       </c>
     </row>
@@ -566,27 +562,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>TCW</t>
+          <t>Strategic Value Partners</t>
         </is>
       </c>
       <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n">
-        <v>62.22</v>
+        <v>83.87</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>pik_stress</t>
+          <t>nav_markdown</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_nav_stability</t>
         </is>
       </c>
     </row>
@@ -596,22 +592,26 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fortress Investment Group</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
+          <t>Sixth Street Partners</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>TSLX</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="n">
-        <v>60.47</v>
+        <v>75</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>lender_fee_compression</t>
+          <t>nav_markdown</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -626,18 +626,18 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Marblegate Asset Management</t>
+          <t>Marathon Asset Management</t>
         </is>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n">
-        <v>60.34</v>
+        <v>72.28</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -656,18 +656,18 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Strategic Value Partners</t>
+          <t>Fortress Investment Group</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n">
-        <v>60</v>
+        <v>67.5</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>lender_fundraise_resilience</t>
+          <t>lender_spread_power</t>
         </is>
       </c>
     </row>
@@ -686,18 +686,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>HPS Investment Partners</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
+          <t>SLR Investment Corp.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>SLRC</t>
+        </is>
+      </c>
       <c r="D7" s="2" t="n">
-        <v>60</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -706,7 +710,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_covenant_tightening</t>
         </is>
       </c>
     </row>
@@ -716,31 +720,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SLR Investment Corp.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>SLRC</t>
-        </is>
-      </c>
+          <t>TCW</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="n">
-        <v>56.05</v>
+        <v>62.69</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>nav_markdown</t>
+          <t>lender_fee_compression</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>lender_fundraise_resilience</t>
+          <t>lender_spread_power</t>
         </is>
       </c>
     </row>
@@ -750,31 +750,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ares Management</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>ASIF</t>
-        </is>
-      </c>
+          <t>HPS Investment Partners</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n">
-        <v>54.97</v>
+        <v>62.12</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>nav_markdown</t>
+          <t>pik_stress</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_nav_stability</t>
         </is>
       </c>
     </row>
@@ -784,26 +780,26 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Brookfield Asset Management</t>
+          <t>Ares Management</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>BAM</t>
+          <t>ASIF</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>53.02</v>
+        <v>58.28</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>pik_stress</t>
+          <t>lender_fee_compression</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -818,22 +814,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Blackstone</t>
+          <t>Partners Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>BCRED</t>
+          <t>PGHN</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>52.03</v>
+        <v>58.11</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>117</v>
+        <v>30</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -842,7 +838,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_nav_stability</t>
         </is>
       </c>
     </row>
@@ -852,31 +848,31 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Apollo Global</t>
+          <t>Brookfield Asset Management</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>ADS</t>
+          <t>BAM</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>51.59</v>
+        <v>56.29</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>redemption_pressure</t>
+          <t>lender_fee_compression</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>lender_fundraise_resilience</t>
+          <t>lender_spread_power</t>
         </is>
       </c>
     </row>
@@ -886,18 +882,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Marathon Asset Management</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n"/>
+          <t>KKR</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>KKR</t>
+        </is>
+      </c>
       <c r="D13" s="2" t="n">
-        <v>49.01</v>
+        <v>52.81</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>74</v>
+        <v>122</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_covenant_tightening</t>
         </is>
       </c>
     </row>
@@ -916,31 +916,31 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Golub Capital</t>
+          <t>Blue Owl Capital</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>OWL</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>48.13</v>
+        <v>48.6</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>nav_markdown</t>
+          <t>redemption_pressure</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>lender_nav_stability</t>
+          <t>lender_fundraise_resilience</t>
         </is>
       </c>
     </row>
@@ -950,31 +950,31 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>KKR</t>
+          <t>Apollo Global</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>KKR</t>
+          <t>ADS</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>47.93</v>
+        <v>48.37</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>pik_stress</t>
+          <t>redemption_pressure</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_fundraise_resilience</t>
         </is>
       </c>
     </row>
@@ -984,22 +984,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Blue Owl Capital</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>OWL</t>
+          <t>BCRED</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>47.3</v>
+        <v>47.9</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>lender_fundraise_resilience</t>
+          <t>lender_spread_power</t>
         </is>
       </c>
     </row>
@@ -1018,31 +1018,31 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>UBS O'Connor</t>
+          <t>Golub Capital</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>47.06</v>
+        <v>46.92</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>8</v>
+        <v>137</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>redemption_pressure</t>
+          <t>nav_markdown</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>lender_fundraise_resilience</t>
+          <t>lender_covenant_tightening</t>
         </is>
       </c>
     </row>
@@ -1061,13 +1061,13 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>43.14</v>
+        <v>44.44</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n">
-        <v>42.59</v>
+        <v>43.37</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>covenant_waiver</t>
+          <t>nav_markdown</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1116,31 +1116,31 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PGIM Private Credit</t>
+          <t>UBS O'Connor</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>PRU</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>39.74</v>
+        <v>36.36</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>nav_markdown</t>
+          <t>redemption_pressure</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>lender_nav_stability</t>
+          <t>lender_fundraise_resilience</t>
         </is>
       </c>
     </row>
@@ -1150,22 +1150,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Sixth Street Partners</t>
+          <t>PGIM Private Credit</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>TSLX</t>
+          <t>PRU</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>30</v>
+        <v>36.05</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>lender_spread_power</t>
+          <t>lender_fundraise_resilience</t>
         </is>
       </c>
     </row>
@@ -1262,24 +1262,24 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>First Brands</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n">
-        <v>62.82</v>
+        <v>84.31</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -1288,24 +1288,28 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>First Brands</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n"/>
+          <t>Informatica</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>INFA</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="n">
-        <v>61.82</v>
+        <v>50</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -1314,24 +1318,28 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Peraton</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
+          <t>Integral Ad Science</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>IAS</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="n">
-        <v>60</v>
+        <v>48.15</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -1340,28 +1348,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Informatica</t>
+          <t>Skillsoft</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>INFA</t>
+          <t>SKIL</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>53.42</v>
+        <v>47.83</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -1370,21 +1378,25 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Medallia</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n"/>
+          <t>Dun &amp; Bradstreet</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>DNB</t>
+        </is>
+      </c>
       <c r="D6" s="2" t="n">
-        <v>51.96</v>
+        <v>45</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>23</v>
@@ -1396,28 +1408,24 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Integral Ad Science</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>IAS</t>
-        </is>
-      </c>
+          <t>Medallia</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n">
-        <v>50.99</v>
+        <v>42.17</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1426,28 +1434,28 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dun &amp; Bradstreet</t>
+          <t>JAMF</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DNB</t>
+          <t>JAMF</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>49.44</v>
+        <v>41.96</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -1456,28 +1464,24 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Skillsoft</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>SKIL</t>
-        </is>
-      </c>
+          <t>Peraton</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n">
-        <v>48.84</v>
+        <v>35</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1486,24 +1490,24 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Conga</t>
+          <t>Zendesk</t>
         </is>
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n">
-        <v>48.48</v>
+        <v>25</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1512,24 +1516,24 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Allego</t>
+          <t>Epicor</t>
         </is>
       </c>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n">
-        <v>47.06</v>
+        <v>22.22</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1538,28 +1542,24 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>JAMF</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>JAMF</t>
-        </is>
-      </c>
+          <t>Cloudera</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n">
-        <v>46.92</v>
+        <v>21.31</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1568,24 +1568,28 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Outreach</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n"/>
+          <t>Instructure</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>INST</t>
+        </is>
+      </c>
       <c r="D13" s="2" t="n">
-        <v>41.67</v>
+        <v>20</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1594,21 +1598,21 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Optimizely</t>
+          <t>Outreach</t>
         </is>
       </c>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="n">
-        <v>41.38</v>
+        <v>19.23</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0</v>
@@ -1620,15 +1624,15 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Seismic</t>
+          <t>Conga</t>
         </is>
       </c>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n">
-        <v>39.66</v>
+        <v>18.6</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>0</v>
@@ -1637,7 +1641,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -1646,24 +1650,24 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Conductor</t>
+          <t>Cision</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n">
-        <v>39.06</v>
+        <v>17.46</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1672,24 +1676,24 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Sitecore</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n">
-        <v>38.98</v>
+        <v>17.14</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1698,25 +1702,21 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Instructure</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>INST</t>
-        </is>
-      </c>
+          <t>Conductor</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n">
-        <v>38.78</v>
+        <v>15.22</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0</v>
@@ -1728,15 +1728,15 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Epicor</t>
+          <t>Sitecore</t>
         </is>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n">
-        <v>38.18</v>
+        <v>13.64</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>0</v>
@@ -1754,21 +1754,21 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Zendesk</t>
+          <t>Seismic</t>
         </is>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n">
-        <v>37.66</v>
+        <v>12.82</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>2</v>
@@ -1780,24 +1780,24 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Cision</t>
+          <t>Cotiviti</t>
         </is>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n">
-        <v>36.26</v>
+        <v>12.5</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1806,21 +1806,21 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Syndigo</t>
+          <t>Allego</t>
         </is>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n">
-        <v>34.85</v>
+        <v>12.2</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>1</v>
@@ -1832,21 +1832,21 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Cotiviti</t>
+          <t>Syndigo</t>
         </is>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n">
-        <v>34.78</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>0</v>
@@ -1858,15 +1858,15 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Solera</t>
+          <t>Optimizely</t>
         </is>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n">
-        <v>33.33</v>
+        <v>5.56</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
@@ -1884,15 +1884,15 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Cloudera</t>
+          <t>Solera</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n">
-        <v>32.05</v>
+        <v>3.33</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -2012,31 +2012,31 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>31</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -2054,25 +2054,25 @@
         <v>31</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G3" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>15</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>24</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>5</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>21</v>
@@ -2090,31 +2090,31 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -2129,7 +2129,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>32</v>
@@ -2141,19 +2141,19 @@
         <v>21</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -2171,28 +2171,28 @@
         <v>31</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>26</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -2203,28 +2203,28 @@
       </c>
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F7" s="2" t="n">
         <v>20</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>19</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>8</v>
@@ -2242,10 +2242,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>5</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
@@ -2281,31 +2281,31 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>19</v>
       </c>
       <c r="E9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>17</v>
-      </c>
       <c r="G9" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>16</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -2323,13 +2323,13 @@
         <v>32</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>30</v>
@@ -2338,13 +2338,13 @@
         <v>31</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
@@ -2359,31 +2359,31 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>17</v>
@@ -2406,19 +2406,19 @@
         <v>18</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -2429,31 +2429,31 @@
       </c>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>6</v>
-      </c>
       <c r="I13" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2464,31 +2464,31 @@
       </c>
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>15</v>
-      </c>
       <c r="F14" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -2503,31 +2503,31 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>3</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2538,13 +2538,13 @@
       </c>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>18</v>
@@ -2553,16 +2553,16 @@
         <v>2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J16" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="K16" s="2" t="n">
         <v>16</v>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -2577,31 +2577,31 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D17" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="F17" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="E17" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>21</v>
-      </c>
       <c r="G17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="I17" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H17" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I17" s="2" t="n">
+      <c r="J17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K17" s="2" t="n">
         <v>11</v>
-      </c>
-      <c r="J17" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="K17" s="2" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="18">
@@ -2612,31 +2612,31 @@
       </c>
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>23</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="K18" s="2" t="n">
         <v>10</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="19">
@@ -2654,10 +2654,10 @@
         <v>6</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>2</v>
@@ -2666,16 +2666,16 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
@@ -2696,16 +2696,16 @@
         <v>8</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I20" s="2" t="n">
         <v>11</v>
@@ -2714,7 +2714,7 @@
         <v>8</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -2725,28 +2725,28 @@
       </c>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>17</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>20</v>
@@ -2928,19 +2928,19 @@
       </c>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>29</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>5</v>
@@ -2949,7 +2949,7 @@
         <v>2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2960,10 +2960,10 @@
       </c>
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
@@ -2972,7 +2972,7 @@
         <v>19</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
@@ -2981,7 +2981,7 @@
         <v>0</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3004,7 +3004,7 @@
         <v>9</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
@@ -3036,16 +3036,16 @@
         <v>21</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3068,7 +3068,7 @@
         <v>15</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>1</v>
@@ -3077,7 +3077,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3091,7 +3091,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -3100,7 +3100,7 @@
         <v>21</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>0</v>
@@ -3123,16 +3123,16 @@
         <v>18</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>20</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>0</v>
@@ -3141,7 +3141,7 @@
         <v>1</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3156,28 +3156,28 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D9" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="I9" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="E9" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>17</v>
-      </c>
       <c r="J9" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -3192,7 +3192,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
@@ -3201,10 +3201,10 @@
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>2</v>
@@ -3233,19 +3233,19 @@
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3260,10 +3260,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>22</v>
@@ -3272,16 +3272,16 @@
         <v>29</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
@@ -3301,10 +3301,10 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>0</v>
@@ -3313,7 +3313,7 @@
         <v>0</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -3331,25 +3331,25 @@
         <v>29</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>10</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -3363,7 +3363,7 @@
         <v>21</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -3372,7 +3372,7 @@
         <v>19</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>3</v>
@@ -3381,7 +3381,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
@@ -3404,7 +3404,7 @@
         <v>8</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>5</v>
@@ -3433,10 +3433,10 @@
         <v>1</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>6</v>
@@ -3445,7 +3445,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -3456,10 +3456,10 @@
       </c>
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -3468,16 +3468,16 @@
         <v>1</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -3495,25 +3495,25 @@
         <v>25</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20">
@@ -3528,10 +3528,10 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>18</v>
@@ -3540,16 +3540,16 @@
         <v>23</v>
       </c>
       <c r="G20" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="J20" s="2" t="n">
         <v>23</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="I20" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="J20" s="2" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="21">
@@ -3563,16 +3563,16 @@
         <v>11</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>0</v>
@@ -3601,10 +3601,10 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>0</v>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>0</v>
@@ -3633,10 +3633,10 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>0</v>
@@ -3645,7 +3645,7 @@
         <v>1</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -3656,25 +3656,25 @@
       </c>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="I24" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0</v>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>1</v>
@@ -3697,10 +3697,10 @@
         <v>1</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Updated to have sentimment filters on pages
</commit_message>
<xml_diff>
--- a/dist/private_credit_stress.xlsx
+++ b/dist/private_credit_stress.xlsx
@@ -3803,7 +3803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -3896,79 +3896,93 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr"/>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Retrieval: each query uses a Bigdata sentiment filter aligned to that topic's polarity</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Scoring Formula:</t>
+          <t xml:space="preserve">  (positive topics favor positive-toned documents; negative topics favor negative-toned).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  terms_power_score = positive_count / (positive_count + negative_count + 1) × 100</t>
-        </is>
-      </c>
+      <c r="A17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  stress_score = 100 - terms_power_score</t>
+          <t>Scoring Formula:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr"/>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  terms_power_score = positive_count / (positive_count + negative_count + 1) × 100</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Layer-Specific Ranking:</t>
+          <t xml:space="preserve">  stress_score = 100 - terms_power_score</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Lenders: ranked by terms_power_score (high = strong)</t>
-        </is>
-      </c>
+      <c r="A21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Borrowers: ranked by stress_score (high = distressed)</t>
+          <t>Layer-Specific Ranking:</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Banks: ranked by net_position = market_share_gain − credit_pullback</t>
+          <t xml:space="preserve">  Lenders: ranked by terms_power_score (high = strong)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr"/>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Borrowers: ranked by stress_score (high = distressed)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Limitations:</t>
+          <t xml:space="preserve">  Banks: ranked by net_position = market_share_gain − credit_pullback</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Scores reflect mention frequency, not sentiment magnitude.</t>
-        </is>
-      </c>
+      <c r="A26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Limitations:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Scores are mention counts after entity-in-text filtering, not chunk sentiment scores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Results depend on Bigdata index coverage and recency.</t>
         </is>

</xml_diff>

<commit_message>
Updated to have overview page
</commit_message>
<xml_diff>
--- a/dist/private_credit_stress.xlsx
+++ b/dist/private_credit_stress.xlsx
@@ -1932,15 +1932,15 @@
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1956,47 +1956,47 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Lender Spread Power</t>
+          <t>Spread power</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Lender Fundraise Resilience</t>
+          <t>Fundraise resilience</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Lender Nav Stability</t>
+          <t>NAV stability</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Lender Covenant Tightening</t>
+          <t>Covenant tightening</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Redemption Pressure</t>
+          <t>Redemption pressure</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>Nav Markdown</t>
+          <t>NAV markdown</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>Covenant Waiver</t>
+          <t>Covenant waiver</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
         <is>
-          <t>Pik Stress</t>
+          <t>PIK stress</t>
         </is>
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Lender Fee Compression</t>
+          <t>Fee compression</t>
         </is>
       </c>
     </row>
@@ -2858,13 +2858,13 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2881,42 +2881,42 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Borrower Revenue Growth</t>
+          <t>Revenue growth</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Borrower Refinancing Success</t>
+          <t>Refinancing success</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Borrower Margin Expansion</t>
+          <t>Margin / EBITDA strength</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Borrower Ai Adoption</t>
+          <t>AI adoption</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Ai Disruption Risk</t>
+          <t>AI disruption risk</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>Maturity Wall</t>
+          <t>Maturity wall</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>Default Risk</t>
+          <t>Default / restructuring</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
         <is>
-          <t>Customer Churn</t>
+          <t>Customer churn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated to have dynamic entities
</commit_message>
<xml_diff>
--- a/dist/private_credit_stress.xlsx
+++ b/dist/private_credit_stress.xlsx
@@ -535,7 +535,9 @@
           <t>Marblegate Asset Management</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
+        <v/>
+      </c>
       <c r="D2" s="2" t="n">
         <v>87.78</v>
       </c>
@@ -565,7 +567,9 @@
           <t>Strategic Value Partners</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="2" t="n">
+        <v/>
+      </c>
       <c r="D3" s="2" t="n">
         <v>83.87</v>
       </c>
@@ -629,7 +633,9 @@
           <t>Marathon Asset Management</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="n">
+        <v/>
+      </c>
       <c r="D5" s="2" t="n">
         <v>72.28</v>
       </c>
@@ -659,7 +665,9 @@
           <t>Fortress Investment Group</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="n">
+        <v/>
+      </c>
       <c r="D6" s="2" t="n">
         <v>67.5</v>
       </c>
@@ -723,7 +731,9 @@
           <t>TCW</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n"/>
+      <c r="C8" s="2" t="n">
+        <v/>
+      </c>
       <c r="D8" s="2" t="n">
         <v>62.69</v>
       </c>
@@ -753,7 +763,9 @@
           <t>HPS Investment Partners</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n"/>
+      <c r="C9" s="2" t="n">
+        <v/>
+      </c>
       <c r="D9" s="2" t="n">
         <v>62.12</v>
       </c>
@@ -1089,7 +1101,9 @@
           <t>AGL Private Credit Income Fund</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n"/>
+      <c r="C19" s="2" t="n">
+        <v/>
+      </c>
       <c r="D19" s="2" t="n">
         <v>43.37</v>
       </c>
@@ -1265,7 +1279,9 @@
           <t>First Brands</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
+        <v/>
+      </c>
       <c r="D2" s="2" t="n">
         <v>84.31</v>
       </c>
@@ -1411,7 +1427,9 @@
           <t>Medallia</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
+      <c r="C7" s="2" t="n">
+        <v/>
+      </c>
       <c r="D7" s="2" t="n">
         <v>42.17</v>
       </c>
@@ -1467,7 +1485,9 @@
           <t>Peraton</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n"/>
+      <c r="C9" s="2" t="n">
+        <v/>
+      </c>
       <c r="D9" s="2" t="n">
         <v>35</v>
       </c>
@@ -1493,7 +1513,9 @@
           <t>Zendesk</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n"/>
+      <c r="C10" s="2" t="n">
+        <v/>
+      </c>
       <c r="D10" s="2" t="n">
         <v>25</v>
       </c>
@@ -1519,7 +1541,9 @@
           <t>Epicor</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n"/>
+      <c r="C11" s="2" t="n">
+        <v/>
+      </c>
       <c r="D11" s="2" t="n">
         <v>22.22</v>
       </c>
@@ -1545,7 +1569,9 @@
           <t>Cloudera</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n"/>
+      <c r="C12" s="2" t="n">
+        <v/>
+      </c>
       <c r="D12" s="2" t="n">
         <v>21.31</v>
       </c>
@@ -1601,7 +1627,9 @@
           <t>Outreach</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n"/>
+      <c r="C14" s="2" t="n">
+        <v/>
+      </c>
       <c r="D14" s="2" t="n">
         <v>19.23</v>
       </c>
@@ -1627,7 +1655,9 @@
           <t>Conga</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n"/>
+      <c r="C15" s="2" t="n">
+        <v/>
+      </c>
       <c r="D15" s="2" t="n">
         <v>18.6</v>
       </c>
@@ -1653,7 +1683,9 @@
           <t>Cision</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n"/>
+      <c r="C16" s="2" t="n">
+        <v/>
+      </c>
       <c r="D16" s="2" t="n">
         <v>17.46</v>
       </c>
@@ -1679,7 +1711,9 @@
           <t>Cornerstone OnDemand</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n"/>
+      <c r="C17" s="2" t="n">
+        <v/>
+      </c>
       <c r="D17" s="2" t="n">
         <v>17.14</v>
       </c>
@@ -1705,7 +1739,9 @@
           <t>Conductor</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n"/>
+      <c r="C18" s="2" t="n">
+        <v/>
+      </c>
       <c r="D18" s="2" t="n">
         <v>15.22</v>
       </c>
@@ -1731,7 +1767,9 @@
           <t>Sitecore</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n"/>
+      <c r="C19" s="2" t="n">
+        <v/>
+      </c>
       <c r="D19" s="2" t="n">
         <v>13.64</v>
       </c>
@@ -1757,7 +1795,9 @@
           <t>Seismic</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n"/>
+      <c r="C20" s="2" t="n">
+        <v/>
+      </c>
       <c r="D20" s="2" t="n">
         <v>12.82</v>
       </c>
@@ -1783,7 +1823,9 @@
           <t>Cotiviti</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n"/>
+      <c r="C21" s="2" t="n">
+        <v/>
+      </c>
       <c r="D21" s="2" t="n">
         <v>12.5</v>
       </c>
@@ -1809,7 +1851,9 @@
           <t>Allego</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n"/>
+      <c r="C22" s="2" t="n">
+        <v/>
+      </c>
       <c r="D22" s="2" t="n">
         <v>12.2</v>
       </c>
@@ -1835,7 +1879,9 @@
           <t>Syndigo</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n"/>
+      <c r="C23" s="2" t="n">
+        <v/>
+      </c>
       <c r="D23" s="2" t="n">
         <v>8.699999999999999</v>
       </c>
@@ -1861,7 +1907,9 @@
           <t>Optimizely</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n"/>
+      <c r="C24" s="2" t="n">
+        <v/>
+      </c>
       <c r="D24" s="2" t="n">
         <v>5.56</v>
       </c>
@@ -1887,7 +1935,9 @@
           <t>Solera</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n"/>
+      <c r="C25" s="2" t="n">
+        <v/>
+      </c>
       <c r="D25" s="2" t="n">
         <v>3.33</v>
       </c>
@@ -2201,7 +2251,9 @@
           <t>HPS Investment Partners</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
+      <c r="B7" s="2" t="n">
+        <v/>
+      </c>
       <c r="C7" s="2" t="n">
         <v>19</v>
       </c>
@@ -2392,7 +2444,9 @@
           <t>Marathon Asset Management</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
+      <c r="B12" s="2" t="n">
+        <v/>
+      </c>
       <c r="C12" s="2" t="n">
         <v>19</v>
       </c>
@@ -2427,7 +2481,9 @@
           <t>Strategic Value Partners</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
+      <c r="B13" s="2" t="n">
+        <v/>
+      </c>
       <c r="C13" s="2" t="n">
         <v>3</v>
       </c>
@@ -2462,7 +2518,9 @@
           <t>Marblegate Asset Management</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n"/>
+      <c r="B14" s="2" t="n">
+        <v/>
+      </c>
       <c r="C14" s="2" t="n">
         <v>21</v>
       </c>
@@ -2536,7 +2594,9 @@
           <t>TCW</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="2" t="n">
+        <v/>
+      </c>
       <c r="C16" s="2" t="n">
         <v>28</v>
       </c>
@@ -2610,7 +2670,9 @@
           <t>Fortress Investment Group</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n"/>
+      <c r="B18" s="2" t="n">
+        <v/>
+      </c>
       <c r="C18" s="2" t="n">
         <v>24</v>
       </c>
@@ -2723,7 +2785,9 @@
           <t>AGL Private Credit Income Fund</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n"/>
+      <c r="B21" s="2" t="n">
+        <v/>
+      </c>
       <c r="C21" s="2" t="n">
         <v>19</v>
       </c>
@@ -2926,7 +2990,9 @@
           <t>Cision</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
+      <c r="B2" s="2" t="n">
+        <v/>
+      </c>
       <c r="C2" s="2" t="n">
         <v>16</v>
       </c>
@@ -2958,7 +3024,9 @@
           <t>Sitecore</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
+      <c r="B3" s="2" t="n">
+        <v/>
+      </c>
       <c r="C3" s="2" t="n">
         <v>18</v>
       </c>
@@ -2990,7 +3058,9 @@
           <t>Optimizely</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n"/>
+      <c r="B4" s="2" t="n">
+        <v/>
+      </c>
       <c r="C4" s="2" t="n">
         <v>8</v>
       </c>
@@ -3022,7 +3092,9 @@
           <t>Conductor</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="n">
+        <v/>
+      </c>
       <c r="C5" s="2" t="n">
         <v>18</v>
       </c>
@@ -3054,7 +3126,9 @@
           <t>Allego</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
+      <c r="B6" s="2" t="n">
+        <v/>
+      </c>
       <c r="C6" s="2" t="n">
         <v>20</v>
       </c>
@@ -3086,7 +3160,9 @@
           <t>Seismic</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
+      <c r="B7" s="2" t="n">
+        <v/>
+      </c>
       <c r="C7" s="2" t="n">
         <v>13</v>
       </c>
@@ -3118,7 +3194,9 @@
           <t>Outreach</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n"/>
+      <c r="B8" s="2" t="n">
+        <v/>
+      </c>
       <c r="C8" s="2" t="n">
         <v>18</v>
       </c>
@@ -3222,7 +3300,9 @@
           <t>Cornerstone OnDemand</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n"/>
+      <c r="B11" s="2" t="n">
+        <v/>
+      </c>
       <c r="C11" s="2" t="n">
         <v>11</v>
       </c>
@@ -3290,7 +3370,9 @@
           <t>Conga</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
+      <c r="B13" s="2" t="n">
+        <v/>
+      </c>
       <c r="C13" s="2" t="n">
         <v>17</v>
       </c>
@@ -3358,7 +3440,9 @@
           <t>Syndigo</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="n">
+        <v/>
+      </c>
       <c r="C15" s="2" t="n">
         <v>21</v>
       </c>
@@ -3390,7 +3474,9 @@
           <t>Peraton</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="2" t="n">
+        <v/>
+      </c>
       <c r="C16" s="2" t="n">
         <v>5</v>
       </c>
@@ -3422,7 +3508,9 @@
           <t>Medallia</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v/>
+      </c>
       <c r="C17" s="2" t="n">
         <v>23</v>
       </c>
@@ -3454,7 +3542,9 @@
           <t>First Brands</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n"/>
+      <c r="B18" s="2" t="n">
+        <v/>
+      </c>
       <c r="C18" s="2" t="n">
         <v>2</v>
       </c>
@@ -3558,7 +3648,9 @@
           <t>Solera</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n"/>
+      <c r="B21" s="2" t="n">
+        <v/>
+      </c>
       <c r="C21" s="2" t="n">
         <v>11</v>
       </c>
@@ -3590,7 +3682,9 @@
           <t>Epicor</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n"/>
+      <c r="B22" s="2" t="n">
+        <v/>
+      </c>
       <c r="C22" s="2" t="n">
         <v>15</v>
       </c>
@@ -3622,7 +3716,9 @@
           <t>Zendesk</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n"/>
+      <c r="B23" s="2" t="n">
+        <v/>
+      </c>
       <c r="C23" s="2" t="n">
         <v>21</v>
       </c>
@@ -3654,7 +3750,9 @@
           <t>Cotiviti</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n"/>
+      <c r="B24" s="2" t="n">
+        <v/>
+      </c>
       <c r="C24" s="2" t="n">
         <v>11</v>
       </c>
@@ -3686,7 +3784,9 @@
           <t>Cloudera</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n"/>
+      <c r="B25" s="2" t="n">
+        <v/>
+      </c>
       <c r="C25" s="2" t="n">
         <v>24</v>
       </c>

</xml_diff>